<commit_message>
Update attendees for quiz: mongodb-second-crew — sharangonsalousj@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -455,9 +455,50 @@
         <v>Grade</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>sharangonsalousj@clarium.tech</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Sharan Gonsalous Johni</v>
+      </c>
+      <c r="C2" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D2" t="str">
+        <v>10/4/2026, 3:55:50 pm</v>
+      </c>
+      <c r="E2">
+        <v>25</v>
+      </c>
+      <c r="F2">
+        <v>25</v>
+      </c>
+      <c r="G2">
+        <v>20</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>41</v>
+      </c>
+      <c r="K2">
+        <v>32</v>
+      </c>
+      <c r="L2" t="str">
+        <v>78.05</v>
+      </c>
+      <c r="M2" t="str">
+        <v>B</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-second-crew — dhatchanamoorthys@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D2" t="str">
-        <v>10/4/2026, 3:55:50 pm</v>
+        <v>10/4/2026, 3:55:50 PM</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -494,11 +494,52 @@
       </c>
       <c r="M2" t="str">
         <v>B</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>dhatchanamoorthys@clarium.tech</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Dhatchanamoorthy</v>
+      </c>
+      <c r="C3" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D3" t="str">
+        <v>4/10/2026, 3:57:33 PM</v>
+      </c>
+      <c r="E3">
+        <v>25</v>
+      </c>
+      <c r="F3">
+        <v>25</v>
+      </c>
+      <c r="G3">
+        <v>20</v>
+      </c>
+      <c r="H3">
+        <v>5</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>41</v>
+      </c>
+      <c r="K3">
+        <v>33</v>
+      </c>
+      <c r="L3" t="str">
+        <v>80.49</v>
+      </c>
+      <c r="M3" t="str">
+        <v>A</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-second-crew — gantasaisirriishaas@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -537,9 +537,50 @@
         <v>A</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>gantasaisirriishaas@clarium.tech</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Ganta Sai Sirriisha</v>
+      </c>
+      <c r="C4" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D4" t="str">
+        <v>4/10/2026, 3:58:49 PM</v>
+      </c>
+      <c r="E4">
+        <v>25</v>
+      </c>
+      <c r="F4">
+        <v>25</v>
+      </c>
+      <c r="G4">
+        <v>21</v>
+      </c>
+      <c r="H4">
+        <v>4</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>41</v>
+      </c>
+      <c r="K4">
+        <v>33</v>
+      </c>
+      <c r="L4" t="str">
+        <v>80.49</v>
+      </c>
+      <c r="M4" t="str">
+        <v>A</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-second-crew — gopikrishnas@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D2" t="str">
-        <v>10/4/2026, 3:55:50 PM</v>
+        <v>4/10/2026, 3:55:50 pm</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D3" t="str">
-        <v>4/10/2026, 3:57:33 PM</v>
+        <v>10/4/2026, 3:57:33 pm</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D4" t="str">
-        <v>4/10/2026, 3:58:49 PM</v>
+        <v>10/4/2026, 3:58:49 pm</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -576,11 +576,52 @@
       </c>
       <c r="M4" t="str">
         <v>A</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>gopikrishnas@clarium.tech</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Gopi Krishna S</v>
+      </c>
+      <c r="C5" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D5" t="str">
+        <v>10/4/2026, 3:59:47 pm</v>
+      </c>
+      <c r="E5">
+        <v>25</v>
+      </c>
+      <c r="F5">
+        <v>25</v>
+      </c>
+      <c r="G5">
+        <v>18</v>
+      </c>
+      <c r="H5">
+        <v>7</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>41</v>
+      </c>
+      <c r="K5">
+        <v>29</v>
+      </c>
+      <c r="L5" t="str">
+        <v>70.73</v>
+      </c>
+      <c r="M5" t="str">
+        <v>B</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-second-crew — karthikeyanm@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D2" t="str">
-        <v>4/10/2026, 3:55:50 pm</v>
+        <v>4/10/2026, 3:55:50 PM</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D3" t="str">
-        <v>10/4/2026, 3:57:33 pm</v>
+        <v>10/4/2026, 3:57:33 PM</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D4" t="str">
-        <v>10/4/2026, 3:58:49 pm</v>
+        <v>10/4/2026, 3:58:49 PM</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -589,7 +589,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D5" t="str">
-        <v>10/4/2026, 3:59:47 pm</v>
+        <v>10/4/2026, 3:59:47 PM</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -617,11 +617,52 @@
       </c>
       <c r="M5" t="str">
         <v>B</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>karthikeyanm@clarium.tech</v>
+      </c>
+      <c r="B6" t="str">
+        <v>karthikeyan</v>
+      </c>
+      <c r="C6" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D6" t="str">
+        <v>4/10/2026, 4:00:49 PM</v>
+      </c>
+      <c r="E6">
+        <v>25</v>
+      </c>
+      <c r="F6">
+        <v>25</v>
+      </c>
+      <c r="G6">
+        <v>22</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>41</v>
+      </c>
+      <c r="K6">
+        <v>35</v>
+      </c>
+      <c r="L6" t="str">
+        <v>85.37</v>
+      </c>
+      <c r="M6" t="str">
+        <v>A</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-second-crew — joyinfantaj@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -660,9 +660,50 @@
         <v>A</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>joyinfantaj@clarium.tech</v>
+      </c>
+      <c r="B7" t="str">
+        <v>joy</v>
+      </c>
+      <c r="C7" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D7" t="str">
+        <v>4/10/2026, 4:01:29 PM</v>
+      </c>
+      <c r="E7">
+        <v>25</v>
+      </c>
+      <c r="F7">
+        <v>25</v>
+      </c>
+      <c r="G7">
+        <v>21</v>
+      </c>
+      <c r="H7">
+        <v>4</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>41</v>
+      </c>
+      <c r="K7">
+        <v>34</v>
+      </c>
+      <c r="L7" t="str">
+        <v>82.93</v>
+      </c>
+      <c r="M7" t="str">
+        <v>A</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-second-crew — harenees@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D2" t="str">
-        <v>4/10/2026, 3:55:50 PM</v>
+        <v>10/4/2026, 3:55:50 pm</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D3" t="str">
-        <v>10/4/2026, 3:57:33 PM</v>
+        <v>4/10/2026, 3:57:33 pm</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D4" t="str">
-        <v>10/4/2026, 3:58:49 PM</v>
+        <v>4/10/2026, 3:58:49 pm</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -589,7 +589,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D5" t="str">
-        <v>10/4/2026, 3:59:47 PM</v>
+        <v>4/10/2026, 3:59:47 pm</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -630,7 +630,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D6" t="str">
-        <v>4/10/2026, 4:00:49 PM</v>
+        <v>10/4/2026, 4:00:49 pm</v>
       </c>
       <c r="E6">
         <v>25</v>
@@ -671,7 +671,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D7" t="str">
-        <v>4/10/2026, 4:01:29 PM</v>
+        <v>10/4/2026, 4:01:29 pm</v>
       </c>
       <c r="E7">
         <v>25</v>
@@ -699,11 +699,52 @@
       </c>
       <c r="M7" t="str">
         <v>A</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>harenees@gmail.com</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Harenee Selvaraj</v>
+      </c>
+      <c r="C8" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D8" t="str">
+        <v>10/4/2026, 4:02:47 pm</v>
+      </c>
+      <c r="E8">
+        <v>25</v>
+      </c>
+      <c r="F8">
+        <v>25</v>
+      </c>
+      <c r="G8">
+        <v>24</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>41</v>
+      </c>
+      <c r="K8">
+        <v>39</v>
+      </c>
+      <c r="L8" t="str">
+        <v>95.12</v>
+      </c>
+      <c r="M8" t="str">
+        <v>A+</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-second-crew — krishnavenikb@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M9"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D2" t="str">
-        <v>10/4/2026, 3:55:50 pm</v>
+        <v>10/4/2026, 3:55:50 PM</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D3" t="str">
-        <v>4/10/2026, 3:57:33 pm</v>
+        <v>4/10/2026, 3:57:33 PM</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D4" t="str">
-        <v>4/10/2026, 3:58:49 pm</v>
+        <v>4/10/2026, 3:58:49 PM</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -589,7 +589,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D5" t="str">
-        <v>4/10/2026, 3:59:47 pm</v>
+        <v>4/10/2026, 3:59:47 PM</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -630,7 +630,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D6" t="str">
-        <v>10/4/2026, 4:00:49 pm</v>
+        <v>10/4/2026, 4:00:49 PM</v>
       </c>
       <c r="E6">
         <v>25</v>
@@ -671,7 +671,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D7" t="str">
-        <v>10/4/2026, 4:01:29 pm</v>
+        <v>10/4/2026, 4:01:29 PM</v>
       </c>
       <c r="E7">
         <v>25</v>
@@ -712,7 +712,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D8" t="str">
-        <v>10/4/2026, 4:02:47 pm</v>
+        <v>10/4/2026, 4:02:47 PM</v>
       </c>
       <c r="E8">
         <v>25</v>
@@ -742,9 +742,50 @@
         <v>A+</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>krishnavenikb@clarium.tech</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Krishnaveni</v>
+      </c>
+      <c r="C9" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D9" t="str">
+        <v>4/10/2026, 4:03:41 PM</v>
+      </c>
+      <c r="E9">
+        <v>25</v>
+      </c>
+      <c r="F9">
+        <v>25</v>
+      </c>
+      <c r="G9">
+        <v>22</v>
+      </c>
+      <c r="H9">
+        <v>3</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>41</v>
+      </c>
+      <c r="K9">
+        <v>36</v>
+      </c>
+      <c r="L9" t="str">
+        <v>87.80</v>
+      </c>
+      <c r="M9" t="str">
+        <v>A</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-second-crew — jebadoss06@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M10"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D2" t="str">
-        <v>10/4/2026, 3:55:50 PM</v>
+        <v>04/10/2026, 15:55:50</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D3" t="str">
-        <v>4/10/2026, 3:57:33 PM</v>
+        <v>10/04/2026, 15:57:33</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D4" t="str">
-        <v>4/10/2026, 3:58:49 PM</v>
+        <v>10/04/2026, 15:58:49</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -589,7 +589,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D5" t="str">
-        <v>4/10/2026, 3:59:47 PM</v>
+        <v>10/04/2026, 15:59:47</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -630,7 +630,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D6" t="str">
-        <v>10/4/2026, 4:00:49 PM</v>
+        <v>04/10/2026, 16:00:49</v>
       </c>
       <c r="E6">
         <v>25</v>
@@ -671,7 +671,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D7" t="str">
-        <v>10/4/2026, 4:01:29 PM</v>
+        <v>04/10/2026, 16:01:29</v>
       </c>
       <c r="E7">
         <v>25</v>
@@ -712,7 +712,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D8" t="str">
-        <v>10/4/2026, 4:02:47 PM</v>
+        <v>04/10/2026, 16:02:47</v>
       </c>
       <c r="E8">
         <v>25</v>
@@ -753,7 +753,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D9" t="str">
-        <v>4/10/2026, 4:03:41 PM</v>
+        <v>10/04/2026, 16:03:41</v>
       </c>
       <c r="E9">
         <v>25</v>
@@ -783,9 +783,50 @@
         <v>A</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>jebadoss06@gmail.com</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Jeba Doss</v>
+      </c>
+      <c r="C10" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D10" t="str">
+        <v>10/04/2026, 16:04:04</v>
+      </c>
+      <c r="E10">
+        <v>25</v>
+      </c>
+      <c r="F10">
+        <v>25</v>
+      </c>
+      <c r="G10">
+        <v>14</v>
+      </c>
+      <c r="H10">
+        <v>11</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>41</v>
+      </c>
+      <c r="K10">
+        <v>21</v>
+      </c>
+      <c r="L10" t="str">
+        <v>51.22</v>
+      </c>
+      <c r="M10" t="str">
+        <v>D</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-second-crew — muthukumarg@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D2" t="str">
-        <v>04/10/2026, 15:55:50</v>
+        <v>4/10/2026, 3:55:50 PM</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D3" t="str">
-        <v>10/04/2026, 15:57:33</v>
+        <v>10/4/2026, 3:57:33 PM</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D4" t="str">
-        <v>10/04/2026, 15:58:49</v>
+        <v>10/4/2026, 3:58:49 PM</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -589,7 +589,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D5" t="str">
-        <v>10/04/2026, 15:59:47</v>
+        <v>10/4/2026, 3:59:47 PM</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -630,7 +630,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D6" t="str">
-        <v>04/10/2026, 16:00:49</v>
+        <v>4/10/2026, 4:00:49 PM</v>
       </c>
       <c r="E6">
         <v>25</v>
@@ -671,7 +671,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D7" t="str">
-        <v>04/10/2026, 16:01:29</v>
+        <v>4/10/2026, 4:01:29 PM</v>
       </c>
       <c r="E7">
         <v>25</v>
@@ -712,7 +712,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D8" t="str">
-        <v>04/10/2026, 16:02:47</v>
+        <v>4/10/2026, 4:02:47 PM</v>
       </c>
       <c r="E8">
         <v>25</v>
@@ -753,7 +753,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D9" t="str">
-        <v>10/04/2026, 16:03:41</v>
+        <v>10/4/2026, 4:03:41 PM</v>
       </c>
       <c r="E9">
         <v>25</v>
@@ -794,7 +794,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D10" t="str">
-        <v>10/04/2026, 16:04:04</v>
+        <v>10/4/2026, 4:04:04 PM</v>
       </c>
       <c r="E10">
         <v>25</v>
@@ -824,9 +824,50 @@
         <v>D</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>muthukumarg@clarium.tech</v>
+      </c>
+      <c r="B11" t="str">
+        <v>MuthukumarG</v>
+      </c>
+      <c r="C11" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D11" t="str">
+        <v>4/10/2026, 4:05:51 PM</v>
+      </c>
+      <c r="E11">
+        <v>25</v>
+      </c>
+      <c r="F11">
+        <v>25</v>
+      </c>
+      <c r="G11">
+        <v>21</v>
+      </c>
+      <c r="H11">
+        <v>4</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>41</v>
+      </c>
+      <c r="K11">
+        <v>34</v>
+      </c>
+      <c r="L11" t="str">
+        <v>82.93</v>
+      </c>
+      <c r="M11" t="str">
+        <v>A</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-second-crew — clementsahayarajm@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M12"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D2" t="str">
-        <v>4/10/2026, 3:55:50 PM</v>
+        <v>10/4/2026, 3:55:50 pm</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D3" t="str">
-        <v>10/4/2026, 3:57:33 PM</v>
+        <v>4/10/2026, 3:57:33 pm</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D4" t="str">
-        <v>10/4/2026, 3:58:49 PM</v>
+        <v>4/10/2026, 3:58:49 pm</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -589,7 +589,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D5" t="str">
-        <v>10/4/2026, 3:59:47 PM</v>
+        <v>4/10/2026, 3:59:47 pm</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -630,7 +630,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D6" t="str">
-        <v>4/10/2026, 4:00:49 PM</v>
+        <v>10/4/2026, 4:00:49 pm</v>
       </c>
       <c r="E6">
         <v>25</v>
@@ -671,7 +671,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D7" t="str">
-        <v>4/10/2026, 4:01:29 PM</v>
+        <v>10/4/2026, 4:01:29 pm</v>
       </c>
       <c r="E7">
         <v>25</v>
@@ -712,7 +712,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D8" t="str">
-        <v>4/10/2026, 4:02:47 PM</v>
+        <v>10/4/2026, 4:02:47 pm</v>
       </c>
       <c r="E8">
         <v>25</v>
@@ -753,7 +753,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D9" t="str">
-        <v>10/4/2026, 4:03:41 PM</v>
+        <v>4/10/2026, 4:03:41 pm</v>
       </c>
       <c r="E9">
         <v>25</v>
@@ -794,7 +794,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D10" t="str">
-        <v>10/4/2026, 4:04:04 PM</v>
+        <v>4/10/2026, 4:04:04 pm</v>
       </c>
       <c r="E10">
         <v>25</v>
@@ -835,7 +835,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D11" t="str">
-        <v>4/10/2026, 4:05:51 PM</v>
+        <v>10/4/2026, 4:05:51 pm</v>
       </c>
       <c r="E11">
         <v>25</v>
@@ -865,9 +865,50 @@
         <v>A</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>clementsahayarajm@clarium.tech</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Clement</v>
+      </c>
+      <c r="C12" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D12" t="str">
+        <v>10/4/2026, 4:06:19 pm</v>
+      </c>
+      <c r="E12">
+        <v>25</v>
+      </c>
+      <c r="F12">
+        <v>25</v>
+      </c>
+      <c r="G12">
+        <v>19</v>
+      </c>
+      <c r="H12">
+        <v>6</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>41</v>
+      </c>
+      <c r="K12">
+        <v>31</v>
+      </c>
+      <c r="L12" t="str">
+        <v>75.61</v>
+      </c>
+      <c r="M12" t="str">
+        <v>B</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-second-crew — suhivasanth04@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D2" t="str">
-        <v>10/4/2026, 3:57:33 pm</v>
+        <v>10/4/2026, 3:57:33 PM</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D3" t="str">
-        <v>10/4/2026, 3:58:49 pm</v>
+        <v>10/4/2026, 3:58:49 PM</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D4" t="str">
-        <v>10/4/2026, 3:59:47 pm</v>
+        <v>10/4/2026, 3:59:47 PM</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -589,7 +589,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D5" t="str">
-        <v>4/10/2026, 4:00:49 pm</v>
+        <v>4/10/2026, 4:00:49 PM</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -630,7 +630,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D6" t="str">
-        <v>4/10/2026, 4:01:29 pm</v>
+        <v>4/10/2026, 4:01:29 PM</v>
       </c>
       <c r="E6">
         <v>25</v>
@@ -671,7 +671,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D7" t="str">
-        <v>4/10/2026, 4:02:47 pm</v>
+        <v>4/10/2026, 4:02:47 PM</v>
       </c>
       <c r="E7">
         <v>25</v>
@@ -712,7 +712,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D8" t="str">
-        <v>10/4/2026, 4:03:41 pm</v>
+        <v>10/4/2026, 4:03:41 PM</v>
       </c>
       <c r="E8">
         <v>25</v>
@@ -753,7 +753,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D9" t="str">
-        <v>10/4/2026, 4:04:04 pm</v>
+        <v>10/4/2026, 4:04:04 PM</v>
       </c>
       <c r="E9">
         <v>25</v>
@@ -794,7 +794,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D10" t="str">
-        <v>4/10/2026, 4:05:51 pm</v>
+        <v>4/10/2026, 4:05:51 PM</v>
       </c>
       <c r="E10">
         <v>25</v>
@@ -835,7 +835,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D11" t="str">
-        <v>4/10/2026, 4:06:19 pm</v>
+        <v>4/10/2026, 4:06:19 PM</v>
       </c>
       <c r="E11">
         <v>25</v>
@@ -876,7 +876,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D12" t="str">
-        <v>10/4/2026, 4:09:04 pm</v>
+        <v>10/4/2026, 4:09:04 PM</v>
       </c>
       <c r="E12">
         <v>25</v>
@@ -906,9 +906,50 @@
         <v>A</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>suhivasanth04@gmail.com</v>
+      </c>
+      <c r="B13" t="str">
+        <v>suhi vasanth</v>
+      </c>
+      <c r="C13" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D13" t="str">
+        <v>4/10/2026, 4:11:17 PM</v>
+      </c>
+      <c r="E13">
+        <v>25</v>
+      </c>
+      <c r="F13">
+        <v>24</v>
+      </c>
+      <c r="G13">
+        <v>10</v>
+      </c>
+      <c r="H13">
+        <v>14</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="J13">
+        <v>41</v>
+      </c>
+      <c r="K13">
+        <v>17</v>
+      </c>
+      <c r="L13" t="str">
+        <v>41.46</v>
+      </c>
+      <c r="M13" t="str">
+        <v>F</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-second-crew — abinayashankar004@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M14"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D2" t="str">
-        <v>10/4/2026, 3:57:33 PM</v>
+        <v>4/10/2026, 3:57:33 pm</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D3" t="str">
-        <v>10/4/2026, 3:58:49 PM</v>
+        <v>4/10/2026, 3:58:49 pm</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D4" t="str">
-        <v>10/4/2026, 3:59:47 PM</v>
+        <v>4/10/2026, 3:59:47 pm</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -589,7 +589,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D5" t="str">
-        <v>4/10/2026, 4:00:49 PM</v>
+        <v>10/4/2026, 4:00:49 pm</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -630,7 +630,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D6" t="str">
-        <v>4/10/2026, 4:01:29 PM</v>
+        <v>10/4/2026, 4:01:29 pm</v>
       </c>
       <c r="E6">
         <v>25</v>
@@ -671,7 +671,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D7" t="str">
-        <v>4/10/2026, 4:02:47 PM</v>
+        <v>10/4/2026, 4:02:47 pm</v>
       </c>
       <c r="E7">
         <v>25</v>
@@ -712,7 +712,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D8" t="str">
-        <v>10/4/2026, 4:03:41 PM</v>
+        <v>4/10/2026, 4:03:41 pm</v>
       </c>
       <c r="E8">
         <v>25</v>
@@ -753,7 +753,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D9" t="str">
-        <v>10/4/2026, 4:04:04 PM</v>
+        <v>4/10/2026, 4:04:04 pm</v>
       </c>
       <c r="E9">
         <v>25</v>
@@ -794,7 +794,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D10" t="str">
-        <v>4/10/2026, 4:05:51 PM</v>
+        <v>10/4/2026, 4:05:51 pm</v>
       </c>
       <c r="E10">
         <v>25</v>
@@ -835,7 +835,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D11" t="str">
-        <v>4/10/2026, 4:06:19 PM</v>
+        <v>10/4/2026, 4:06:19 pm</v>
       </c>
       <c r="E11">
         <v>25</v>
@@ -876,7 +876,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D12" t="str">
-        <v>10/4/2026, 4:09:04 PM</v>
+        <v>4/10/2026, 4:09:04 pm</v>
       </c>
       <c r="E12">
         <v>25</v>
@@ -917,7 +917,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D13" t="str">
-        <v>4/10/2026, 4:13:31 PM</v>
+        <v>10/4/2026, 4:13:31 pm</v>
       </c>
       <c r="E13">
         <v>25</v>
@@ -947,9 +947,50 @@
         <v>F</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>abinayashankar004@gmail.com</v>
+      </c>
+      <c r="B14" t="str">
+        <v>abinaya</v>
+      </c>
+      <c r="C14" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D14" t="str">
+        <v>10/4/2026, 4:12:39 pm</v>
+      </c>
+      <c r="E14">
+        <v>25</v>
+      </c>
+      <c r="F14">
+        <v>25</v>
+      </c>
+      <c r="G14">
+        <v>15</v>
+      </c>
+      <c r="H14">
+        <v>10</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>41</v>
+      </c>
+      <c r="K14">
+        <v>24</v>
+      </c>
+      <c r="L14" t="str">
+        <v>58.54</v>
+      </c>
+      <c r="M14" t="str">
+        <v>D</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-second-crew — srimathitech1@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D2" t="str">
-        <v>4/10/2026, 3:57:33 pm</v>
+        <v>4/10/2026, 3:57:33 PM</v>
       </c>
       <c r="E2">
         <v>25</v>
@@ -507,7 +507,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D3" t="str">
-        <v>4/10/2026, 3:58:49 pm</v>
+        <v>4/10/2026, 3:58:49 PM</v>
       </c>
       <c r="E3">
         <v>25</v>
@@ -548,7 +548,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D4" t="str">
-        <v>4/10/2026, 3:59:47 pm</v>
+        <v>4/10/2026, 3:59:47 PM</v>
       </c>
       <c r="E4">
         <v>25</v>
@@ -589,7 +589,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D5" t="str">
-        <v>10/4/2026, 4:00:49 pm</v>
+        <v>10/4/2026, 4:00:49 PM</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -630,7 +630,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D6" t="str">
-        <v>10/4/2026, 4:01:29 pm</v>
+        <v>10/4/2026, 4:01:29 PM</v>
       </c>
       <c r="E6">
         <v>25</v>
@@ -671,7 +671,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D7" t="str">
-        <v>10/4/2026, 4:02:47 pm</v>
+        <v>10/4/2026, 4:02:47 PM</v>
       </c>
       <c r="E7">
         <v>25</v>
@@ -712,7 +712,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D8" t="str">
-        <v>4/10/2026, 4:03:41 pm</v>
+        <v>4/10/2026, 4:03:41 PM</v>
       </c>
       <c r="E8">
         <v>25</v>
@@ -753,7 +753,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D9" t="str">
-        <v>4/10/2026, 4:04:04 pm</v>
+        <v>4/10/2026, 4:04:04 PM</v>
       </c>
       <c r="E9">
         <v>25</v>
@@ -794,7 +794,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D10" t="str">
-        <v>10/4/2026, 4:05:51 pm</v>
+        <v>10/4/2026, 4:05:51 PM</v>
       </c>
       <c r="E10">
         <v>25</v>
@@ -835,7 +835,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D11" t="str">
-        <v>10/4/2026, 4:06:19 pm</v>
+        <v>10/4/2026, 4:06:19 PM</v>
       </c>
       <c r="E11">
         <v>25</v>
@@ -876,7 +876,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D12" t="str">
-        <v>4/10/2026, 4:09:04 pm</v>
+        <v>4/10/2026, 4:09:04 PM</v>
       </c>
       <c r="E12">
         <v>25</v>
@@ -917,7 +917,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D13" t="str">
-        <v>10/4/2026, 4:13:31 pm</v>
+        <v>10/4/2026, 4:13:31 PM</v>
       </c>
       <c r="E13">
         <v>25</v>
@@ -958,7 +958,7 @@
         <v>MongoDB Second Crew</v>
       </c>
       <c r="D14" t="str">
-        <v>10/4/2026, 4:12:39 pm</v>
+        <v>10/4/2026, 4:12:39 PM</v>
       </c>
       <c r="E14">
         <v>25</v>
@@ -988,9 +988,50 @@
         <v>D</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>srimathitech1@gmail.com</v>
+      </c>
+      <c r="B15" t="str">
+        <v>srimathi srimathi</v>
+      </c>
+      <c r="C15" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D15" t="str">
+        <v>4/10/2026, 4:12:59 PM</v>
+      </c>
+      <c r="E15">
+        <v>25</v>
+      </c>
+      <c r="F15">
+        <v>25</v>
+      </c>
+      <c r="G15">
+        <v>18</v>
+      </c>
+      <c r="H15">
+        <v>7</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>41</v>
+      </c>
+      <c r="K15">
+        <v>29</v>
+      </c>
+      <c r="L15" t="str">
+        <v>70.73</v>
+      </c>
+      <c r="M15" t="str">
+        <v>B</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: mongodb-second-crew — kajamoideena@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/mongodb-second-crew/attendees.xlsx
+++ b/quizzes/mongodb-second-crew/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M16"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -1029,9 +1029,50 @@
         <v>B</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>kajamoideena@clarium.tech</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Kajamoideen Abbas</v>
+      </c>
+      <c r="C16" t="str">
+        <v>MongoDB Second Crew</v>
+      </c>
+      <c r="D16" t="str">
+        <v>4/10/2026, 4:37:44 PM</v>
+      </c>
+      <c r="E16">
+        <v>25</v>
+      </c>
+      <c r="F16">
+        <v>25</v>
+      </c>
+      <c r="G16">
+        <v>23</v>
+      </c>
+      <c r="H16">
+        <v>2</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>41</v>
+      </c>
+      <c r="K16">
+        <v>38</v>
+      </c>
+      <c r="L16" t="str">
+        <v>92.68</v>
+      </c>
+      <c r="M16" t="str">
+        <v>A+</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>